<commit_message>
Convertir plantilla a Tabla de Excel para agregar filas facilmente
</commit_message>
<xml_diff>
--- a/Plantilla_Cotizacion_Proveedor.xlsx
+++ b/Plantilla_Cotizacion_Proveedor.xlsx
@@ -16,8 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="_-$* #,##0.00_-;-$* #,##0.00_-;_-$* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,24 +38,13 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="006E152E"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -93,14 +84,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -178,6 +169,20 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TablaCotizacion" displayName="TablaCotizacion" ref="A6:E16" headerRowCount="1">
+  <autoFilter ref="A6:E16"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Partida"/>
+    <tableColumn id="2" name="Descripcion"/>
+    <tableColumn id="3" name="Cantidad"/>
+    <tableColumn id="4" name="Precio_Unitario"/>
+    <tableColumn id="5" name="Importe"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -469,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -518,7 +523,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Descripcion del Servicio / Bien</t>
+          <t>Descripcion</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -528,7 +533,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Precio Unitario</t>
+          <t>Precio_Unitario</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -538,158 +543,131 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="4">
-        <f>IF(ISNUMBER(C7),C7*D7,"")</f>
+        <f>IF(ISNUMBER($C7),$C7*$D7,"")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="4">
-        <f>IF(ISNUMBER(C8),C8*D8,"")</f>
+        <f>IF(ISNUMBER($C8),$C8*$D8,"")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4">
-        <f>IF(ISNUMBER(C9),C9*D9,"")</f>
+        <f>IF(ISNUMBER($C9),$C9*$D9,"")</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n"/>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="4">
-        <f>IF(ISNUMBER(C10),C10*D10,"")</f>
+        <f>IF(ISNUMBER($C10),$C10*$D10,"")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="4">
-        <f>IF(ISNUMBER(C11),C11*D11,"")</f>
+        <f>IF(ISNUMBER($C11),$C11*$D11,"")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="4">
-        <f>IF(ISNUMBER(C12),C12*D12,"")</f>
+        <f>IF(ISNUMBER($C12),$C12*$D12,"")</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="4">
-        <f>IF(ISNUMBER(C13),C13*D13,"")</f>
+        <f>IF(ISNUMBER($C13),$C13*$D13,"")</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="4">
-        <f>IF(ISNUMBER(C14),C14*D14,"")</f>
+        <f>IF(ISNUMBER($C14),$C14*$D14,"")</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="4">
-        <f>IF(ISNUMBER(C15),C15*D15,"")</f>
+        <f>IF(ISNUMBER($C15),$C15*$D15,"")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4">
-        <f>IF(ISNUMBER(C16),C16*D16,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Subtotal:</t>
-        </is>
-      </c>
-      <c r="E17" s="6">
-        <f>SUM(E7:E16)</f>
+        <f>IF(ISNUMBER($C16),$C16*$D16,"")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>IVA 16%:</t>
+          <t>Subtotal:</t>
         </is>
       </c>
       <c r="E18" s="6">
-        <f>E17*0.16</f>
+        <f>SUM(TablaCotizacion[Importe])</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="D19" s="5" t="inlineStr">
         <is>
+          <t>IVA 16%:</t>
+        </is>
+      </c>
+      <c r="E19" s="6">
+        <f>E18*0.16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" s="5" t="inlineStr">
+        <is>
           <t>Total:</t>
         </is>
       </c>
-      <c r="E19" s="6">
-        <f>E17+E18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>__________________________________________________</t>
-        </is>
+      <c r="E20" s="6">
+        <f>E18+E19</f>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="7" t="inlineStr">
         <is>
+          <t>__________________________________________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
           <t>Nombre y Firma del Representante Legal</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B25:D25"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B24:D24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajustar colores corporativos y area de impresion tamaño carta
</commit_message>
<xml_diff>
--- a/Plantilla_Cotizacion_Proveedor.xlsx
+++ b/Plantilla_Cotizacion_Proveedor.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-$* #,##0.00_-;-$* #,##0.00_-;_-$* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,8 +38,14 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,17 +54,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="006E152E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EBE2D1"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <bottom style="hair">
+        <color rgb="00CCCCCC"/>
+      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -78,22 +94,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -176,12 +193,12 @@
   <autoFilter ref="A6:E16"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Partida"/>
-    <tableColumn id="2" name="Descripcion"/>
+    <tableColumn id="2" name="Descripcion del Servicio o Bien"/>
     <tableColumn id="3" name="Cantidad"/>
-    <tableColumn id="4" name="Precio_Unitario"/>
+    <tableColumn id="4" name="Precio Unitario"/>
     <tableColumn id="5" name="Importe"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -472,19 +489,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>FORMATO ESTANDARIZADO DE COTIZACION COMERCIAL</t>
@@ -523,7 +540,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Descripcion</t>
+          <t>Descripcion del Servicio o Bien</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -533,7 +550,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Precio_Unitario</t>
+          <t>Precio Unitario</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -543,117 +560,147 @@
       </c>
     </row>
     <row r="7">
-      <c r="D7" s="4" t="n"/>
-      <c r="E7" s="4">
+      <c r="A7" s="4" t="n"/>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5">
         <f>IF(ISNUMBER($C7),$C7*$D7,"")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4">
+      <c r="A8" s="4" t="n"/>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5">
         <f>IF(ISNUMBER($C8),$C8*$D8,"")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4">
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5">
         <f>IF(ISNUMBER($C9),$C9*$D9,"")</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4">
+      <c r="A10" s="4" t="n"/>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5">
         <f>IF(ISNUMBER($C10),$C10*$D10,"")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4">
+      <c r="A11" s="4" t="n"/>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5">
         <f>IF(ISNUMBER($C11),$C11*$D11,"")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4">
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5">
         <f>IF(ISNUMBER($C12),$C12*$D12,"")</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4">
+      <c r="A13" s="4" t="n"/>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5">
         <f>IF(ISNUMBER($C13),$C13*$D13,"")</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5">
         <f>IF(ISNUMBER($C14),$C14*$D14,"")</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5">
         <f>IF(ISNUMBER($C15),$C15*$D15,"")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5">
         <f>IF(ISNUMBER($C16),$C16*$D16,"")</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Subtotal:</t>
         </is>
       </c>
-      <c r="E18" s="6">
+      <c r="E18" s="7">
         <f>SUM(TablaCotizacion[Importe])</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>IVA 16%:</t>
         </is>
       </c>
-      <c r="E19" s="6">
+      <c r="E19" s="7">
         <f>E18*0.16</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>Total:</t>
         </is>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="7">
         <f>E18+E19</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="7" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>__________________________________________________</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="7" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Nombre y Firma del Representante Legal</t>
         </is>
@@ -661,11 +708,13 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="B26:D26"/>
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B24:D24"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="1" right="1" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Intercalar colores de la tabla usando tonos institucionales
</commit_message>
<xml_diff>
--- a/Plantilla_Cotizacion_Proveedor.xlsx
+++ b/Plantilla_Cotizacion_Proveedor.xlsx
@@ -116,6 +116,15 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00EBE2D1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -712,6 +721,11 @@
     <mergeCell ref="B25:D25"/>
     <mergeCell ref="A1:E1"/>
   </mergeCells>
+  <conditionalFormatting sqref="A7:E16">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Agregar hoja de instrucciones claras para los proveedores
</commit_message>
<xml_diff>
--- a/Plantilla_Cotizacion_Proveedor.xlsx
+++ b/Plantilla_Cotizacion_Proveedor.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cotizacion" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cotizacion" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-$* #,##0.00_-;-$* #,##0.00_-;_-$* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +33,16 @@
       <b val="1"/>
       <color rgb="006E152E"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -94,22 +105,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -498,6 +515,97 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>GUIA PARA EL LLENADO DE LA COTIZACION COMERCIAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="5">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>1. LLENADO DIGITAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="65" customHeight="1">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>• Ingrese los datos de su empresa (Proveedor), Fecha, Moneda y Vigencia en la parte superior de la hoja 'Cotizacion'.
+• Llene unicamente las columnas de 'Cantidad' y 'Precio Unitario'. La columna de 'Importe' y los totales (Subtotal, IVA, Total) se calcularan automaticamente.
+• Si requiere agregar mas conceptos, ubiquese en la ultima fila de la tabla y presione la tecla 'Tab' (o clic derecho &gt; Insertar Fila). Las formulas y colores se ajustaran solos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2. IMPRESION</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="65" customHeight="1">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>• Una vez capturados todos los datos, proceda a imprimir unicamente la hoja llamada 'Cotizacion'.
+• La hoja ya se encuentra pre-configurada para imprimirse correctamente en hoja Tamano Carta (Letter) sin que los margenes se corten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>3. FIRMA AUTOGRAFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="65" customHeight="1">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>• El documento impreso debe ser firmado de manera autografa en la parte inferior (Nombre y Firma del Representante Legal).
+• Si cuenta con sello oficial de la empresa, anexelo a un costado de la firma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>4. ESCANEO Y ENVIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="65" customHeight="1">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>• Escanee el documento ya firmado y guardelo en formato PDF.
+• Asegurese de que el escaneo sea a color, con buena iluminacion y sin inclinaciones pronunciadas (evite tomar fotografias con el celular de ser posible, priorice un escaner plano).
+• Envie el archivo PDF final al correo institucional que le haya sido indicado.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:B3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:E26"/>
@@ -518,198 +626,198 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Proveedor:</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Moneda (MXN/USD/EUR):</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Fecha:</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Vigencia de cotizacion:</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Partida</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Descripcion del Servicio o Bien</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Precio Unitario</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Importe</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7">
         <f>IF(ISNUMBER($C7),$C7*$D7,"")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n"/>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7">
         <f>IF(ISNUMBER($C8),$C8*$D8,"")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7">
         <f>IF(ISNUMBER($C9),$C9*$D9,"")</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n"/>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7">
         <f>IF(ISNUMBER($C10),$C10*$D10,"")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7">
         <f>IF(ISNUMBER($C11),$C11*$D11,"")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="7">
         <f>IF(ISNUMBER($C12),$C12*$D12,"")</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="7">
         <f>IF(ISNUMBER($C13),$C13*$D13,"")</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="5" t="n"/>
-      <c r="E14" s="5">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7">
         <f>IF(ISNUMBER($C14),$C14*$D14,"")</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7">
         <f>IF(ISNUMBER($C15),$C15*$D15,"")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7">
         <f>IF(ISNUMBER($C16),$C16*$D16,"")</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Subtotal:</t>
         </is>
       </c>
-      <c r="E18" s="7">
+      <c r="E18" s="9">
         <f>SUM(TablaCotizacion[Importe])</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="D19" s="6" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>IVA 16%:</t>
         </is>
       </c>
-      <c r="E19" s="7">
+      <c r="E19" s="9">
         <f>E18*0.16</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Total:</t>
         </is>
       </c>
-      <c r="E20" s="7">
+      <c r="E20" s="9">
         <f>E18+E19</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>__________________________________________________</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Nombre y Firma del Representante Legal</t>
         </is>

</xml_diff>

<commit_message>
Agregar detalle aclaratorio de cada columna en hoja de instrucciones
</commit_message>
<xml_diff>
--- a/Plantilla_Cotizacion_Proveedor.xlsx
+++ b/Plantilla_Cotizacion_Proveedor.xlsx
@@ -517,11 +517,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B15"/>
+  <dimension ref="B2:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -535,61 +535,79 @@
     <row r="5">
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1. LLENADO DIGITAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="65" customHeight="1">
+          <t>1. INSTRUCCIONES GENERALES</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>• Ingrese los datos de su empresa (Proveedor), Fecha, Moneda y Vigencia en la parte superior de la hoja 'Cotizacion'.
-• Llene unicamente las columnas de 'Cantidad' y 'Precio Unitario'. La columna de 'Importe' y los totales (Subtotal, IVA, Total) se calcularan automaticamente.
-• Si requiere agregar mas conceptos, ubiquese en la ultima fila de la tabla y presione la tecla 'Tab' (o clic derecho &gt; Insertar Fila). Las formulas y colores se ajustaran solos.</t>
+• Llene unicamente las celdas permitidas. Los totales (Subtotal, IVA, Total) se calcularan automaticamente.
+• Si requiere agregar mas conceptos, ubiquese en la ultima fila de la tabla y presione la tecla 'Tab' (o clic derecho &gt; Insertar Fila).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2. IMPRESION</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="65" customHeight="1">
+          <t>2. DETALLE DE LAS COLUMNAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="100" customHeight="1">
       <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>• Partida: Numero consecutivo (ej. 1, 2, 3...) o numero de referencia tecnica si la dependencia se lo solicito previamente.
+• Descripcion del Servicio o Bien: Descripcion clara y detallada del producto o servicio que esta cotizando.
+• Cantidad: Numero total de unidades a cotizar. Ingrese unicamente numeros.
+• Precio Unitario: Costo unitario del bien/servicio ANTES de impuestos. Ingrese solo el numero, el formato de moneda ($) se aplicara solo.
+• Importe: NO ESCRIBIR NADA. Esta celda tiene formula y se calcula automaticamente multiplicando la Cantidad por el Precio Unitario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>3. IMPRESION</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>• Una vez capturados todos los datos, proceda a imprimir unicamente la hoja llamada 'Cotizacion'.
 • La hoja ya se encuentra pre-configurada para imprimirse correctamente en hoja Tamano Carta (Letter) sin que los margenes se corten.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>3. FIRMA AUTOGRAFA</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="65" customHeight="1">
-      <c r="B12" s="3" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>4. FIRMA AUTOGRAFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>• El documento impreso debe ser firmado de manera autografa en la parte inferior (Nombre y Firma del Representante Legal).
 • Si cuenta con sello oficial de la empresa, anexelo a un costado de la firma.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>4. ESCANEO Y ENVIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="65" customHeight="1">
-      <c r="B15" s="3" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>5. ESCANEO Y ENVIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>• Escanee el documento ya firmado y guardelo en formato PDF.
-• Asegurese de que el escaneo sea a color, con buena iluminacion y sin inclinaciones pronunciadas (evite tomar fotografias con el celular de ser posible, priorice un escaner plano).
+• Asegurese de que el escaneo sea a color, con buena iluminacion y sin inclinaciones pronunciadas (priorice usar un escaner plano, evite fotos de celular).
 • Envie el archivo PDF final al correo institucional que le haya sido indicado.</t>
         </is>
       </c>

</xml_diff>